<commit_message>
sync(data): operations 答案修正 + 题目附件 + 理论flag/最近作答/错题归档 migration
从主仓库 trainer 同步:
- data/operations.json 答案与模板修正
- 题目附件(ipynb/xlsx)更新
- 新增 migration 020/021/022(自动按 glob 顺序执行)
不含任何运行时/真实数据;classes.json 保持空版。
</commit_message>
<xml_diff>
--- a/data/questions/19/大学生低碳生活行为的影响因素数据集.xlsx
+++ b/data/questions/19/大学生低碳生活行为的影响因素数据集.xlsx
@@ -4,7 +4,9 @@
   <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="27628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15"/>
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\"/>
+    </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8905AA-DC69-4326-B844-685A2331EEB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>

</xml_diff>